<commit_message>
Give the built-but-unreachable features their screens
Batch one of the screen backlog: eleven screens, mostly endpoints that were
finished months apart from any way to open them.

The biggest is the child's own file. Fees, documents, library loans and
conduct were school-wide registers you filtered by hand, even though every
one of those endpoints already took a student_id - so the question staff are
actually asked at a counter, about one child, took four screens to answer.
They are now tabs on that child, with a new per-child attendance history
behind the first one.

Also wired: signing off a paper's marks (the four-eyes check the backend
enforces had no button), the asset assignment register, the settings and
integrations index, a host confirming a visitor, and a library members list
that answers the counter question - can this person take another book.

170 of 296 screens now stand up, from 160.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/School_ERP_296_Development_Tracker.xlsx
+++ b/School_ERP_296_Development_Tracker.xlsx
@@ -9298,9 +9298,9 @@
           <t>Ready</t>
         </is>
       </c>
-      <c r="J66" s="38" t="inlineStr">
-        <is>
-          <t>In progress</t>
+      <c r="J66" s="33" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K66" s="33" t="inlineStr">
@@ -9332,7 +9332,7 @@
       <c r="Q66" s="24" t="n"/>
       <c r="R66" s="24" t="inlineStr">
         <is>
-          <t>Aggregate counts only; no per-child history</t>
+          <t>Attendance tab: months, percent and days away</t>
         </is>
       </c>
       <c r="S66" s="24" t="n"/>
@@ -9506,9 +9506,9 @@
           <t>Ready</t>
         </is>
       </c>
-      <c r="J68" s="38" t="inlineStr">
-        <is>
-          <t>In progress</t>
+      <c r="J68" s="33" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K68" s="33" t="inlineStr">
@@ -9540,7 +9540,7 @@
       <c r="Q68" s="24" t="n"/>
       <c r="R68" s="24" t="inlineStr">
         <is>
-          <t>Cannot scope the fee list to one child</t>
+          <t>Fees tab scoped to the child</t>
         </is>
       </c>
       <c r="S68" s="24" t="n"/>
@@ -9572,7 +9572,7 @@
       </c>
       <c r="AB68" t="inlineStr">
         <is>
-          <t>/school/fees</t>
+          <t>/school/students/[id]</t>
         </is>
       </c>
     </row>
@@ -9610,9 +9610,9 @@
           <t>Ready</t>
         </is>
       </c>
-      <c r="J69" s="38" t="inlineStr">
-        <is>
-          <t>In progress</t>
+      <c r="J69" s="33" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K69" s="33" t="inlineStr">
@@ -9644,7 +9644,7 @@
       <c r="Q69" s="24" t="n"/>
       <c r="R69" s="24" t="inlineStr">
         <is>
-          <t>No per-student document view</t>
+          <t>Documents tab with download</t>
         </is>
       </c>
       <c r="S69" s="24" t="n"/>
@@ -9676,7 +9676,7 @@
       </c>
       <c r="AB69" t="inlineStr">
         <is>
-          <t>/school/documents</t>
+          <t>/school/students/[id]</t>
         </is>
       </c>
     </row>
@@ -9714,9 +9714,9 @@
           <t>Ready</t>
         </is>
       </c>
-      <c r="J70" s="38" t="inlineStr">
-        <is>
-          <t>In progress</t>
+      <c r="J70" s="33" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K70" s="33" t="inlineStr">
@@ -9748,7 +9748,7 @@
       <c r="Q70" s="24" t="n"/>
       <c r="R70" s="24" t="inlineStr">
         <is>
-          <t>Discipline list filters status, not student</t>
+          <t>Conduct tab: incidents for this child</t>
         </is>
       </c>
       <c r="S70" s="24" t="n"/>
@@ -9780,7 +9780,7 @@
       </c>
       <c r="AB70" t="inlineStr">
         <is>
-          <t>/school/discipline</t>
+          <t>/school/students/[id]</t>
         </is>
       </c>
     </row>
@@ -10026,9 +10026,9 @@
           <t>Ready</t>
         </is>
       </c>
-      <c r="J73" s="38" t="inlineStr">
-        <is>
-          <t>In progress</t>
+      <c r="J73" s="33" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K73" s="33" t="inlineStr">
@@ -10060,7 +10060,7 @@
       <c r="Q73" s="24" t="n"/>
       <c r="R73" s="24" t="inlineStr">
         <is>
-          <t>Circulation desk, not a per-student view</t>
+          <t>Library tab: loans, overdue and fines</t>
         </is>
       </c>
       <c r="S73" s="24" t="n"/>
@@ -10092,7 +10092,7 @@
       </c>
       <c r="AB73" t="inlineStr">
         <is>
-          <t>/school/library</t>
+          <t>/school/students/[id]</t>
         </is>
       </c>
     </row>
@@ -18450,9 +18450,9 @@
           <t>Ready</t>
         </is>
       </c>
-      <c r="J154" s="39" t="inlineStr">
-        <is>
-          <t>Not started</t>
+      <c r="J154" s="33" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K154" s="33" t="inlineStr">
@@ -18484,7 +18484,7 @@
       <c r="Q154" s="24" t="n"/>
       <c r="R154" s="24" t="inlineStr">
         <is>
-          <t>Verify endpoint has no caller in the frontend</t>
+          <t>Sign off a paper; refuses whoever entered the marks</t>
         </is>
       </c>
       <c r="S154" s="24" t="n"/>
@@ -18516,7 +18516,7 @@
       </c>
       <c r="AB154" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>/school/exams</t>
         </is>
       </c>
     </row>
@@ -23962,14 +23962,14 @@
           <t>Ready</t>
         </is>
       </c>
-      <c r="J207" s="39" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="K207" s="38" t="inlineStr">
-        <is>
-          <t>In progress</t>
+      <c r="J207" s="33" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K207" s="33" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="L207" s="24" t="inlineStr">
@@ -23996,7 +23996,7 @@
       <c r="Q207" s="24" t="n"/>
       <c r="R207" s="24" t="inlineStr">
         <is>
-          <t>No members screen; borrowers only a picker</t>
+          <t>Who holds what, with limit and can-borrow</t>
         </is>
       </c>
       <c r="S207" s="24" t="n"/>
@@ -24028,7 +24028,7 @@
       </c>
       <c r="AB207" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>/school/library/members</t>
         </is>
       </c>
     </row>
@@ -26770,9 +26770,9 @@
           <t>Ready</t>
         </is>
       </c>
-      <c r="J234" s="38" t="inlineStr">
-        <is>
-          <t>In progress</t>
+      <c r="J234" s="33" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K234" s="33" t="inlineStr">
@@ -26804,7 +26804,7 @@
       <c r="Q234" s="24" t="n"/>
       <c r="R234" s="24" t="inlineStr">
         <is>
-          <t>Host-decision endpoint has no screen</t>
+          <t>Host confirms or declines an expected visitor</t>
         </is>
       </c>
       <c r="S234" s="24" t="n"/>
@@ -28018,9 +28018,9 @@
           <t>Ready</t>
         </is>
       </c>
-      <c r="J246" s="38" t="inlineStr">
-        <is>
-          <t>In progress</t>
+      <c r="J246" s="33" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="K246" s="33" t="inlineStr">
@@ -28052,7 +28052,7 @@
       <c r="Q246" s="24" t="n"/>
       <c r="R246" s="24" t="inlineStr">
         <is>
-          <t>Per asset only; assignments register unused</t>
+          <t>Assignments tab: what is out and with whom</t>
         </is>
       </c>
       <c r="S246" s="24" t="n"/>
@@ -33119,9 +33119,9 @@
           <t>Done</t>
         </is>
       </c>
-      <c r="K295" s="38" t="inlineStr">
-        <is>
-          <t>In progress</t>
+      <c r="K295" s="33" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="L295" s="24" t="inlineStr">
@@ -33148,7 +33148,7 @@
       <c r="Q295" s="24" t="n"/>
       <c r="R295" s="24" t="inlineStr">
         <is>
-          <t>Settings hub endpoint unused</t>
+          <t>Settings index with set-up state</t>
         </is>
       </c>
       <c r="S295" s="24" t="n"/>
@@ -33180,7 +33180,7 @@
       </c>
       <c r="AB295" t="inlineStr">
         <is>
-          <t>/school/profile</t>
+          <t>/school/settings</t>
         </is>
       </c>
     </row>
@@ -33426,14 +33426,14 @@
           <t>Ready</t>
         </is>
       </c>
-      <c r="J298" s="38" t="inlineStr">
-        <is>
-          <t>In progress</t>
-        </is>
-      </c>
-      <c r="K298" s="38" t="inlineStr">
-        <is>
-          <t>In progress</t>
+      <c r="J298" s="33" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K298" s="33" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="L298" s="24" t="inlineStr">
@@ -33460,7 +33460,7 @@
       <c r="Q298" s="24" t="n"/>
       <c r="R298" s="24" t="inlineStr">
         <is>
-          <t>Razorpay keys only; integrations endpoint unused</t>
+          <t>Outside services and whether they are connected</t>
         </is>
       </c>
       <c r="S298" s="24" t="n"/>
@@ -33492,7 +33492,7 @@
       </c>
       <c r="AB298" t="inlineStr">
         <is>
-          <t>/school/fees/online</t>
+          <t>/school/settings</t>
         </is>
       </c>
     </row>

</xml_diff>